<commit_message>
Update project pages, reports and code downloads
</commit_message>
<xml_diff>
--- a/projects/medication-identity/downloads/medication_identity_results.xlsx
+++ b/projects/medication-identity/downloads/medication_identity_results.xlsx
@@ -16441,8 +16441,10 @@
           <t>52817-822-50</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>52817082250</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>52817082250</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -16469,8 +16471,10 @@
           <t>0143-1268-10</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>143126810</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00143126810</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -16497,8 +16501,10 @@
           <t>61919-909-30</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>61919090930</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>61919090930</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -16525,8 +16531,10 @@
           <t>0002-7512-01</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>2751201</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>00002751201</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -16553,8 +16561,10 @@
           <t>0002-7512-99</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>2751299</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>00002751299</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -16581,8 +16591,10 @@
           <t>0002-7510-99</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>2751099</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>00002751099</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -16609,8 +16621,10 @@
           <t>0002-8208-01</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>2820801</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>00002820801</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -16637,8 +16651,10 @@
           <t>0002-8208-27</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>2820827</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>00002820827</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -16660,8 +16676,10 @@
           <t>0002-8799-61</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>2879961</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>00002879961</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -16688,8 +16706,10 @@
           <t>71656-017-16</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>71656001716</v>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>71656001716</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -16716,8 +16736,10 @@
           <t>71656-017-50</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>71656001750</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>71656001750</t>
+        </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -16744,8 +16766,10 @@
           <t>71656-017-51</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>71656001751</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>71656001751</t>
+        </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -16772,8 +16796,10 @@
           <t>71656-017-52</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>71656001752</v>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>71656001752</t>
+        </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>

</xml_diff>